<commit_message>
feat(secret-guard): P04 MVP — AI-path secrets scan CLI
Zero-dep scanner for CLAUDE.md, .cursor/rules, MCP env, .env.example
with redacted findings, --json/--sarif, and pre-commit exit codes.
Patterns specialized from setup-doctor; suite maps updated.
</commit_message>
<xml_diff>
--- a/Software_Opportunity_Research_Portfolio.xlsx
+++ b/Software_Opportunity_Research_Portfolio.xlsx
@@ -1765,12 +1765,12 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Building</t>
         </is>
       </c>
       <c r="P8" s="14" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>MVP CLI</t>
         </is>
       </c>
       <c r="Q8" s="14" t="inlineStr">
@@ -1790,7 +1790,7 @@
       </c>
       <c r="T8" s="15" t="inlineStr">
         <is>
-          <t>Can extract patterns from setup-doctor secret checks</t>
+          <t>Local package ai-secret-guard@0.1.0-beta.0; scan AI paths + MCP env + SARIF; co-located at development/secret-guard</t>
         </is>
       </c>
       <c r="U8" s="14" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>MVP CLI</t>
         </is>
       </c>
       <c r="F10" s="31" t="inlineStr">

</xml_diff>

<commit_message>
feat(portfolio): P05–P28 offline MVPs + suite litmus harness
Scaffold domain cores for all products through P28 with litmus tests,
demos, and cross-fixtures. Add suite-litmus (retry) and suite-watch
scheduler. Update README/CLAUDE/portfolio/memory. No remote push.
</commit_message>
<xml_diff>
--- a/Software_Opportunity_Research_Portfolio.xlsx
+++ b/Software_Opportunity_Research_Portfolio.xlsx
@@ -1860,12 +1860,12 @@
       </c>
       <c r="O9" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P10" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q10" s="14" t="inlineStr">
@@ -2050,12 +2050,12 @@
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
@@ -2145,12 +2145,12 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P12" s="14" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q12" s="14" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P14" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q14" s="14" t="inlineStr">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="O15" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P15" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q15" s="9" t="inlineStr">
@@ -2525,12 +2525,12 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P16" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q16" s="14" t="inlineStr">
@@ -2620,12 +2620,12 @@
       </c>
       <c r="O17" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P17" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q17" s="9" t="inlineStr">
@@ -2715,12 +2715,12 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P18" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q18" s="14" t="inlineStr">
@@ -2810,12 +2810,12 @@
       </c>
       <c r="O19" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P19" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q19" s="9" t="inlineStr">
@@ -2905,12 +2905,12 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P20" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q20" s="14" t="inlineStr">
@@ -3000,12 +3000,12 @@
       </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P21" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q21" s="9" t="inlineStr">
@@ -3095,12 +3095,12 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P22" s="14" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q22" s="14" t="inlineStr">
@@ -3190,12 +3190,12 @@
       </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P23" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q23" s="9" t="inlineStr">
@@ -3285,12 +3285,12 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P24" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q24" s="14" t="inlineStr">
@@ -3380,12 +3380,12 @@
       </c>
       <c r="O25" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P25" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q25" s="9" t="inlineStr">
@@ -3475,12 +3475,12 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P26" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q26" s="14" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="O27" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P27" s="9" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q27" s="9" t="inlineStr">
@@ -3665,12 +3665,12 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P28" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q28" s="14" t="inlineStr">
@@ -3760,12 +3760,12 @@
       </c>
       <c r="O29" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P29" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q29" s="9" t="inlineStr">
@@ -3855,12 +3855,12 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P30" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q30" s="14" t="inlineStr">
@@ -3950,12 +3950,12 @@
       </c>
       <c r="O31" s="9" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P31" s="9" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q31" s="9" t="inlineStr">
@@ -4045,12 +4045,12 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Concept</t>
+          <t>Scaffolded MVP</t>
         </is>
       </c>
       <c r="P32" s="14" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="Q32" s="14" t="inlineStr">
@@ -12890,7 +12890,7 @@
       </c>
       <c r="E16" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="E17" s="34" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F17" s="34" t="inlineStr">
@@ -12960,7 +12960,7 @@
       </c>
       <c r="E18" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F18" s="34" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr">
@@ -13030,7 +13030,7 @@
       </c>
       <c r="E20" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F20" s="34" t="inlineStr">
@@ -13100,7 +13100,7 @@
       </c>
       <c r="E22" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F22" s="34" t="inlineStr">
@@ -13135,7 +13135,7 @@
       </c>
       <c r="E23" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F23" s="34" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="E24" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F24" s="34" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="E25" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F25" s="34" t="inlineStr">
@@ -13240,7 +13240,7 @@
       </c>
       <c r="E26" s="34" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F26" s="34" t="inlineStr">
@@ -13275,7 +13275,7 @@
       </c>
       <c r="E27" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F27" s="34" t="inlineStr">
@@ -13310,7 +13310,7 @@
       </c>
       <c r="E28" s="34" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F28" s="34" t="inlineStr">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="E29" s="34" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F29" s="34" t="inlineStr">
@@ -13465,7 +13465,7 @@
       </c>
       <c r="E35" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F35" s="37" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="E36" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F36" s="37" t="inlineStr">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="E37" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F37" s="37" t="inlineStr">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="E38" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F38" s="37" t="inlineStr">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="E39" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F39" s="37" t="inlineStr">
@@ -13640,7 +13640,7 @@
       </c>
       <c r="E40" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F40" s="37" t="inlineStr">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="E41" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F41" s="37" t="inlineStr">
@@ -13710,7 +13710,7 @@
       </c>
       <c r="E42" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F42" s="37" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="E43" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F43" s="37" t="inlineStr">
@@ -13780,7 +13780,7 @@
       </c>
       <c r="E44" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F44" s="37" t="inlineStr">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="E45" s="37" t="inlineStr">
         <is>
-          <t>Watch</t>
+          <t>Offline MVP + litmus</t>
         </is>
       </c>
       <c r="F45" s="37" t="inlineStr">

</xml_diff>

<commit_message>
docs: portfolio Alpha/Beta cycle-closed statuses
</commit_message>
<xml_diff>
--- a/Software_Opportunity_Research_Portfolio.xlsx
+++ b/Software_Opportunity_Research_Portfolio.xlsx
@@ -1765,12 +1765,12 @@
       </c>
       <c r="O8" s="14" t="inlineStr">
         <is>
-          <t>Building</t>
+          <t>Beta (cycle closed)</t>
         </is>
       </c>
       <c r="P8" s="14" t="inlineStr">
         <is>
-          <t>MVP CLI</t>
+          <t>Beta closed — local</t>
         </is>
       </c>
       <c r="Q8" s="14" t="inlineStr">
@@ -1860,12 +1860,12 @@
       </c>
       <c r="O9" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P9" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q9" s="9" t="inlineStr">
@@ -1955,12 +1955,12 @@
       </c>
       <c r="O10" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P10" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q10" s="14" t="inlineStr">
@@ -2050,12 +2050,12 @@
       </c>
       <c r="O11" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P11" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q11" s="9" t="inlineStr">
@@ -2145,12 +2145,12 @@
       </c>
       <c r="O12" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P12" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q12" s="14" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q13" s="9" t="inlineStr">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="O14" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P14" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q14" s="14" t="inlineStr">
@@ -2430,12 +2430,12 @@
       </c>
       <c r="O15" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P15" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q15" s="9" t="inlineStr">
@@ -2525,12 +2525,12 @@
       </c>
       <c r="O16" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P16" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q16" s="14" t="inlineStr">
@@ -2620,12 +2620,12 @@
       </c>
       <c r="O17" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P17" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q17" s="9" t="inlineStr">
@@ -2715,12 +2715,12 @@
       </c>
       <c r="O18" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P18" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q18" s="14" t="inlineStr">
@@ -2810,12 +2810,12 @@
       </c>
       <c r="O19" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P19" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q19" s="9" t="inlineStr">
@@ -2905,12 +2905,12 @@
       </c>
       <c r="O20" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P20" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q20" s="14" t="inlineStr">
@@ -3000,12 +3000,12 @@
       </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P21" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q21" s="9" t="inlineStr">
@@ -3095,12 +3095,12 @@
       </c>
       <c r="O22" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P22" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q22" s="14" t="inlineStr">
@@ -3190,12 +3190,12 @@
       </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P23" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q23" s="9" t="inlineStr">
@@ -3285,12 +3285,12 @@
       </c>
       <c r="O24" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P24" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q24" s="14" t="inlineStr">
@@ -3380,12 +3380,12 @@
       </c>
       <c r="O25" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P25" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q25" s="9" t="inlineStr">
@@ -3475,12 +3475,12 @@
       </c>
       <c r="O26" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P26" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q26" s="14" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="O27" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P27" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q27" s="9" t="inlineStr">
@@ -3665,12 +3665,12 @@
       </c>
       <c r="O28" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P28" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q28" s="14" t="inlineStr">
@@ -3760,12 +3760,12 @@
       </c>
       <c r="O29" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P29" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q29" s="9" t="inlineStr">
@@ -3855,12 +3855,12 @@
       </c>
       <c r="O30" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P30" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q30" s="14" t="inlineStr">
@@ -3950,12 +3950,12 @@
       </c>
       <c r="O31" s="9" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P31" s="9" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q31" s="9" t="inlineStr">
@@ -4045,12 +4045,12 @@
       </c>
       <c r="O32" s="14" t="inlineStr">
         <is>
-          <t>Scaffolded MVP</t>
+          <t>Alpha (cycle closed)</t>
         </is>
       </c>
       <c r="P32" s="14" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="Q32" s="14" t="inlineStr">
@@ -12770,7 +12770,7 @@
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
-          <t>MVP CLI</t>
+          <t>Beta closed — local</t>
         </is>
       </c>
       <c r="F10" s="31" t="inlineStr">
@@ -12890,7 +12890,7 @@
       </c>
       <c r="E16" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F16" s="34" t="inlineStr">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="E17" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F17" s="34" t="inlineStr">
@@ -12960,7 +12960,7 @@
       </c>
       <c r="E18" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F18" s="34" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr">
@@ -13030,7 +13030,7 @@
       </c>
       <c r="E20" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F20" s="34" t="inlineStr">
@@ -13100,7 +13100,7 @@
       </c>
       <c r="E22" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F22" s="34" t="inlineStr">
@@ -13135,7 +13135,7 @@
       </c>
       <c r="E23" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F23" s="34" t="inlineStr">
@@ -13170,7 +13170,7 @@
       </c>
       <c r="E24" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F24" s="34" t="inlineStr">
@@ -13205,7 +13205,7 @@
       </c>
       <c r="E25" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F25" s="34" t="inlineStr">
@@ -13240,7 +13240,7 @@
       </c>
       <c r="E26" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F26" s="34" t="inlineStr">
@@ -13275,7 +13275,7 @@
       </c>
       <c r="E27" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F27" s="34" t="inlineStr">
@@ -13310,7 +13310,7 @@
       </c>
       <c r="E28" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F28" s="34" t="inlineStr">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="E29" s="34" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F29" s="34" t="inlineStr">
@@ -13465,7 +13465,7 @@
       </c>
       <c r="E35" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F35" s="37" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="E36" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F36" s="37" t="inlineStr">
@@ -13535,7 +13535,7 @@
       </c>
       <c r="E37" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F37" s="37" t="inlineStr">
@@ -13570,7 +13570,7 @@
       </c>
       <c r="E38" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F38" s="37" t="inlineStr">
@@ -13605,7 +13605,7 @@
       </c>
       <c r="E39" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F39" s="37" t="inlineStr">
@@ -13640,7 +13640,7 @@
       </c>
       <c r="E40" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F40" s="37" t="inlineStr">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="E41" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F41" s="37" t="inlineStr">
@@ -13710,7 +13710,7 @@
       </c>
       <c r="E42" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F42" s="37" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="E43" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F43" s="37" t="inlineStr">
@@ -13780,7 +13780,7 @@
       </c>
       <c r="E44" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F44" s="37" t="inlineStr">
@@ -13815,7 +13815,7 @@
       </c>
       <c r="E45" s="37" t="inlineStr">
         <is>
-          <t>Offline MVP + litmus</t>
+          <t>Alpha closed — litmus+cycle</t>
         </is>
       </c>
       <c r="F45" s="37" t="inlineStr">

</xml_diff>